<commit_message>
feat: polish ModelGuard merge review
</commit_message>
<xml_diff>
--- a/public/samples/modelguard-version-1.xlsx
+++ b/public/samples/modelguard-version-1.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="84">
   <si>
     <t>ModelGuard Clean Sample</t>
   </si>
@@ -844,14 +844,12 @@
         <v>23</v>
       </c>
       <c r="B10" s="4">
-        <v>0.09</v>
+        <v>0.07</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D10" s="4" t="s">
-        <v>11</v>
-      </c>
+      <c r="D10" s="4"/>
       <c r="E10" s="4" t="s">
         <v>12</v>
       </c>
@@ -867,7 +865,7 @@
         <v>25</v>
       </c>
       <c r="B11" s="4">
-        <v>0.025</v>
+        <v>0.08</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>10</v>
@@ -1007,8 +1005,7 @@
         <v>1000</v>
       </c>
       <c r="C5">
-        <f>=B5*(1+Inputs!$B$5)</f>
-        <v>1080</v>
+        <v>1190</v>
       </c>
       <c r="D5">
         <f>=C5*(1+Inputs!$B$5)</f>

</xml_diff>